<commit_message>
[CF-Pages-Skip] Update D1 Excel export
</commit_message>
<xml_diff>
--- a/scripts/data_export.xlsx
+++ b/scripts/data_export.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Main'!$A$1:$F$119</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'gdrives'!$A$1:$B$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'images'!$A$1:$B$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'links'!$A$1:$C$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'links'!$A$1:$C$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1556,7 +1556,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Kayansh</t>
+          <t>Kavyansh</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -4083,7 +4083,7 @@
   <dimension ref="A1:B77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -4654,6 +4654,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Amey</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>https://lh4.googleusercontent.com/J0agiE5dHnjO2Z3jxKKkWuixUq7YAMtXpYbxo1ffjP7aH_lyuZu5T9rbKhAIUPG-Tso=w2400</t>
         </is>
       </c>
@@ -4661,6 +4666,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>Anjali</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/g65k5DJtlZ5LFzrfkX44hj1D4tDQu3OKcSu3S9BF0IK9AudCbHcGqsHk0Ghhcg530cI=w2400</t>
         </is>
       </c>
@@ -4668,6 +4678,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>Annu</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/geDJ7KQRVr3-Yb2pUgRx2tgaffeaSm9eXnpCzkazQVw-KgOlPDi8UzJf98v2ZMtyPK8=w2400</t>
         </is>
       </c>
@@ -4675,6 +4690,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Anushka</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/bFBQj1jIvkkWSS2XmxCXkJ1oswyRC5GizER0gtUp3UEtx6nAm6errW3xrPFGpqUlLrM=w2400</t>
         </is>
       </c>
@@ -4682,6 +4702,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Aparna2</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/_sitcZvUG0m2TEbwqaVT2YJ0krvOrimtP4a5QRopqdYQKCxs5WzeHK6b-wF0vxhGTwE=w2400</t>
         </is>
       </c>
@@ -4689,6 +4714,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>Ashlesha</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/lAvIpY0feBCaOvjIjONQrIUfmAZWoCgpSGsZaW5VCJG2PpWlU-4GeD7bvlp0LZLPrck=w2400</t>
         </is>
       </c>
@@ -4696,6 +4726,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>Atulchandra</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/iHWiRa7vzQ7rekxCjafFg1OcZWmBLq3uPuzA0p4nnkuZF7_ICGmuyGd7qWKsL89rtNg=w2400</t>
         </is>
       </c>
@@ -4703,6 +4738,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>Bhalchandra</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/H7cW6B0j_M68TSBsgT4mj5wRzJ60eJ0-XjjjwGSIrR6KFF5uGg5QnMJuE5kFmU7UvkE=w2400</t>
         </is>
       </c>
@@ -4710,6 +4750,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Chandrashekhar2</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/xy7iZE1Fx5gkTMvxDvGV0She3i-Zx8zVeen7CboC9ypO0HnugvHjNygLErDKiu0SPrY=w2400</t>
         </is>
       </c>
@@ -4717,6 +4762,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>Geetanjali</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/PVS5pRq605q2RZy4dbqiWKYJKgqMjDn_y2siLJ8kbaW7rARc-8vSLktzgR_NltgDiU8=w2400</t>
         </is>
       </c>
@@ -4724,6 +4774,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>Jyoti</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/35ufQu_Wfw8QGJj9F5X-KZXwcO0cyTcircMQK4G2JrMh74IAcZXim-v4Ku1ui2Gdq6M=w2400</t>
         </is>
       </c>
@@ -4731,6 +4786,11 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>Kamala</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/69F7Myd5ZVkBAEaVQHJuIr8GI0I9gK4d-UGMRqTwTNRoJZJvX0TtKRwN2ZUa8X7Mm1k=w2400</t>
         </is>
       </c>
@@ -4738,6 +4798,11 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>Kanchan</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/wS6kk5KvNMIYyk8Gk64vuhOQfwzwQKz60CYJjrssRTXbluR_lQvZo6DD_sILKxcv7dQ=w2400</t>
         </is>
       </c>
@@ -4745,6 +4810,11 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
+          <t>Mangala</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/cIdCdDvnjujh1Z3a_CAtmtIVDKwWyofix6T08EO6wGoZ3fyG5q2G6yEj1POwvx7PSXs=w2400</t>
         </is>
       </c>
@@ -4752,6 +4822,11 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>Neeta</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/Ci__EfFDGo3Ns3CFNUaktQn5sncCk222f-fNKmkPla5vYoMnqdmTihkv4F9qGbE1FBo=w2400</t>
         </is>
       </c>
@@ -4759,6 +4834,11 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>Prakash</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/IiR01JebM8ePwMioSgXhcE-ImHq2dWKyABhY_gcSC98wEk38Uz6hXHf7-fND3vQlHfo=w2400</t>
         </is>
       </c>
@@ -4766,6 +4846,11 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>Pratap</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/AVy7lAl4c_lJ2lqy1JiX8_VLhC6_iKJas049Lnfk1W_xNvvB6zpByKS6ZqwiVvgYUR0=w2400</t>
         </is>
       </c>
@@ -4773,6 +4858,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
+          <t>Radha</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/awXPfgABA8fsqNJpfTZTpxfM69c6qdmpSinxmethEV4vsLhSCsDLwJUs1nkzcJ9h6vU=w2400</t>
         </is>
       </c>
@@ -4780,6 +4870,11 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>Radhika</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/oTTxfqK5rKpwTz3ENbzCR2lbg21MXzKPaHllgRHp_aT4ZwLwElK2_vi4G-IrB0krx44=w2400</t>
         </is>
       </c>
@@ -4787,6 +4882,11 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
+          <t>Rajendra</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/9_H1pqB7sJGpQ80MnVeuJF53kfeJKe9uxeVsQecMAUBV7O07EGy15nWkORq1UyvNPGg=w2400</t>
         </is>
       </c>
@@ -4794,6 +4894,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>Renuka</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/1vyAG_0MfdaOWRws918WjYmavq_o6R9XBwdrnmv0Galr98mw4dGSSAomoC8to0v0D3M=w2400</t>
         </is>
       </c>
@@ -4801,6 +4906,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>Rohini</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/zHGycwOP4QjcmHOVd3Dvf-QVqrdwK5gKnAAZHSvY2KdlNg0LPy_1KOvrgV4pKGKDOQg=w2400</t>
         </is>
       </c>
@@ -4808,6 +4918,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>Ruta</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/h8-M28b7ZecHWRRMbMBNBIx6DnRUxm_14LUI5KjbIQg86svsZAwI1rYEraQlXRNt9wU=w2400</t>
         </is>
       </c>
@@ -4815,6 +4930,11 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>Sanjay</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
           <t>https://lh3.googleusercontent.com/yxS2nh4DT-3ZyxE_B5cROmbaFDKh4Aaib6idA-28CJAUTUl15bH_pdepZL2AjwRG4t8=w2400</t>
         </is>
       </c>
@@ -4822,6 +4942,11 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>Sudhir</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>https://lh4.googleusercontent.com/3Kx0sxALtB7PK_KCM9zEjZaMSVESzkNbcZ6OasFsOBl58OASUQw4Pceqr69WQZOnpTc=w2400</t>
         </is>
       </c>
@@ -4829,6 +4954,11 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>Suhasini</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/My53J2599tVpB-4k6mjhn3cWnyGp6LvgWFsMB-pO3KBymBc4okEOli9Ffods_NXSAs0=w2400</t>
         </is>
       </c>
@@ -4836,6 +4966,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>Varsha</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/xMUxxQ4M7TkCr4rIMxPOD3xluROVzxIBuxLTbGgdlaljYnCiEzWCFWvMk1xmEg7D4Sc=w2400</t>
         </is>
       </c>
@@ -4843,6 +4978,11 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>Vidyadhar</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
           <t>https://lh6.googleusercontent.com/iMGuVRci8w51EvsCgcnC9jG153EGlnBj6uVRnvEF8lPdgMunigjU0wQ6RNQiTCdFZK0=w2400</t>
         </is>
       </c>
@@ -4850,12 +4990,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>Vidyadhar2</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
           <t>https://lh5.googleusercontent.com/g10f_me4f5ZwjPsy21iGrD3c_UKy7pIibPjvABvBKiJ17Xp_tn3KNLS-YXa5A5_dCII=w2400</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
+        <is>
+          <t>Vrunda</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
         <is>
           <t>https://lh4.googleusercontent.com/gcqkWsidqISDG1kbdW-SPpK8GiCmIBiVF-Ei3ypG_QELNQW5TVhY2hbK-8hjpWngS5s=w2400</t>
         </is>
@@ -4873,12 +5023,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4894,7 +5044,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>tooltip</t>
         </is>
       </c>
     </row>
@@ -4909,11 +5059,7 @@
           <t>https://mr.wikipedia.org/wiki/%E0%A4%AD%E0%A4%BE%E0%A4%B8%E0%A5%8D%E0%A4%95%E0%A4%B0%E0%A4%B0%E0%A4%BE%E0%A4%B5_%E0%A4%A6%E0%A5%81%E0%A4%B0%E0%A5%8D%E0%A4%B5%E0%A5%87</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>wiki</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4926,11 +5072,7 @@
           <t>https://drive.google.com/file/d/14WLWW9JhhwiLrifUw549d-YNgnoxJOBZ/view?usp=share_link</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>&lt;img src="https://lh6.googleusercontent.com/dbLenSJLpL1qJO9fZEQZenlTIt3PnjXwNyVEwp8rnIg0CUxNEmYDNmQ8dhoTdAdfUew=w2400" alt="Nayak.jpg" width="40" height="40"&gt;</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4943,11 +5085,7 @@
           <t>https://en.wikipedia.org/wiki/Bhai_Vaidya</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>wiki</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4960,11 +5098,7 @@
           <t>https://en.wikipedia.org/wiki/Sohil_Vaidya</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>wiki</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4977,11 +5111,7 @@
           <t>https://www.instagram.com/sohilvaidya/?hl=en</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>instagram</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4994,11 +5124,7 @@
           <t>https://indianexpress.com/article/cities/pune/pune-residents-student-film-about-graffiti-artists-wins-top-honour-at-dga-awards-5503299/</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Indian Express 21/12/2018</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -5011,11 +5137,7 @@
           <t>https://vimeo.com/205442395</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Geeta Film by Sohil</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5028,11 +5150,7 @@
           <t>https://mitwpu.edu.in/campuslife/dr-aparna-watve</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MITWPU</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5045,11 +5163,7 @@
           <t>https://scholar.google.com/citations?user=klf2_rsAAAAJ&amp;hl=en</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Google Scholar</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5062,11 +5176,7 @@
           <t>https://www.researchgate.net/profile/Aparna-Watve</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Researchgate</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5079,11 +5189,7 @@
           <t>https://era-india.org/community/aparna-vidyadhar-watve/</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Ecological Reasearch Alliance</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5096,11 +5202,7 @@
           <t>https://www.flickr.com/photos/sushamadurve/</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Pictures drawn</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -5113,11 +5215,7 @@
           <t>https://www.funkyrainbow.com/03-illustrator/sushama-durve/</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Pictures drawn</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -5130,11 +5228,7 @@
           <t>https://jpip.org/sujala-watve/</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>JPIP</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5147,11 +5241,7 @@
           <t>https://www.instagram.com/sujalawatve/?hl=en</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>instagram</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5164,11 +5254,7 @@
           <t>https://www.justdial.com/Pune/Dr-Vidyadhar-G-Watve-Poona-Hospital-Research-Centre-Near-Alka-Cinema-Sadashiv-Peth/020PXX20-XX20-160108115046-O6Q1_BZDET</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>PHRC</t>
-        </is>
-      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5181,11 +5267,7 @@
           <t>https://www.linkedin.com/in/vidyadhar-watve-453117a5/?originalSubdomain=in</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5198,14 +5280,49 @@
           <t>https://intotomorrow.com/tag/pushkar-durve/</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Infotomorrow with Dave Graveline</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Nakul</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://github.com/nakuldurve-web/family-tree-web</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sanjiv</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://github.com/sbdurve/family-tree-web</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Annu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1coU7gI6gazZaztf4bxQXJ-KEsc-8dGz4?usp=share_link</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C19"/>
+  <autoFilter ref="A1:C22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>